<commit_message>
driggs: add annual operating-cost view to build-out model
Adds a 'what does it cost to RUN the place' annual carrying-cost estimate at
the end of each phase, as a new Operating Cost tab in the xlsx plus a section
in the md. Categories: property tax, insurance (WUI), utilities, snow removal,
internet, trash, servicing, upkeep reserve, optional caretaking.

Likely all-in: ~$23k/yr Phase 1, ~$56k/yr Phase 2 (~$38k cash). Tax + insurance
+ upkeep reserve dominate and scale with value built; utilities stay modest
(well/septic/solar). Notes Teton Co.'s low effective rate (~0.35-0.5%), the
Idaho ag-valuation retention lever (63-604, gated on CC&Rs allowing ag use),
and WUI insurance as the escalating risk.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xxu7aLEZbdzmUJPZjmgRxA
</commit_message>
<xml_diff>
--- a/driggs/construction-estimate.xlsx
+++ b/driggs/construction-estimate.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Cost Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operating Cost" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,6 +108,18 @@
       <color rgb="005F6B70"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005F6B70"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -167,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -229,6 +242,26 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -325,6 +358,26 @@
     <comment ref="D34" authorId="0" shapeId="0">
       <text>
         <t>$500 simple/efficient to $750 sleek w/ big glass. Single-story adds cost per sf.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>estimate</author>
+  </authors>
+  <commentList>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Median effective rate in Teton County is 0.35%. A full-market second home with no homeowner exemption pays the levy rate; 0.5% is a reasonable planning midpoint.</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>Idaho §63-604: platting alone doesn't end ag status. Keep the balance in qualifying ag use (&gt;5 ac, $1,000+ ag revenue) and it stays ag-valued — UNLESS CC&amp;Rs prohibit ag use.</t>
       </text>
     </comment>
   </commentList>
@@ -1211,8 +1264,466 @@
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Annual Operating Cost — What It Costs to RUN the Place</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>First-estimate carrying cost at the end of each phase. 2026 dollars. Edit blue cells. See notes at right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>TAX &amp; RESERVE ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Effective property-tax rate</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Teton Co. median effective 0.35%; use 0.5% for a full-market second home. Verify w/ Treasurer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Assessed improvements — end of Phase 1</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>ADU + garage market value (~build cost proxy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Assessed improvements — end of Phase 2</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>+ main house; total improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Assessed homesite land (taxed portion)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>~1 ac at market IF the balance stays ag-valued (§63-604). Whole parcel ~$500k if not farmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Major repair/replacement reserve</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>% of improvement value set aside yearly for roof/siding/systems (sinking fund, not cash spent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ANNUAL COST</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>(end of phase)</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>ADU + garage</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>full build-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Property tax</t>
+        </is>
+      </c>
+      <c r="C13" s="17">
+        <f>(C6+C8)*C5</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>(C7+C8)*C5</f>
+        <v/>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Low rate, but scales with what's built</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Insurance (WUI / high-value)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Wildfire-exposed; market hardening — a real risk line</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Electricity (Fall River, net of solar)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>$39/mo access fee; solar offsets much of the geo load</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Propane (cooking / backup / fireplace)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Optional; minimal if fully electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Internet (Starlink / rural)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>~$120/mo; same both phases</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Trash / recycling</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Rural hauler or county transfer station</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Snow removal (driveway)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Long rural drive, heavy Teton snow, all winter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Shared road maintenance</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Crossed Arrows road easement (per CC&amp;Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Landscape / defensible space</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>WUI defensible-space upkeep; low-maint. design helps</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Well / septic / HVAC servicing</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>700</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Septic pump ~3–5 yr; well &amp; geo annual service</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Cash operating subtotal</t>
+        </is>
+      </c>
+      <c r="C23" s="19">
+        <f>SUM(C13:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>SUM(D13:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Major repair/replacement reserve</t>
+        </is>
+      </c>
+      <c r="C24" s="17">
+        <f>C6*C9</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>C7*C9</f>
+        <v/>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Sinking fund for long-cycle replacements</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Caretaking / property mgmt (if 2nd home)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Optional; winter check-ins for an absentee home</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>TOTAL ALL-IN / YEAR</t>
+        </is>
+      </c>
+      <c r="C26" s="28">
+        <f>C23+C24+C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="28">
+        <f>D23+D24+D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="27" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>≈ per month</t>
+        </is>
+      </c>
+      <c r="C27" s="35">
+        <f>C26/12</f>
+        <v/>
+      </c>
+      <c r="D27" s="35">
+        <f>D26/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>Cash-only (excl. reserve &amp; caretaking)</t>
+        </is>
+      </c>
+      <c r="C29" s="37">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="D29" s="37">
+        <f>D23</f>
+        <v/>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>What actually leaves your pocket each year</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56" customHeight="1">
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>First-estimate only. The big three — property tax, insurance, and the maintenance reserve — all scale with the VALUE of what's built, so Phase 2 roughly triples the carrying cost even though the utility bills stay modest (well + septic + solar = no water/sewer bill and a small net electric bill). Verify the tax rate &amp; assessed value with the Teton County Assessor/Treasurer, get a real insurance quote (WUI underwriting is tightening), and confirm ag-valuation retention against the CC&amp;Rs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
driggs: add annual operating-cost view to build-out model (#28)
Adds a 'what does it cost to RUN the place' annual carrying-cost estimate at
the end of each phase, as a new Operating Cost tab in the xlsx plus a section
in the md. Categories: property tax, insurance (WUI), utilities, snow removal,
internet, trash, servicing, upkeep reserve, optional caretaking.

Likely all-in: ~$23k/yr Phase 1, ~$56k/yr Phase 2 (~$38k cash). Tax + insurance
+ upkeep reserve dominate and scale with value built; utilities stay modest
(well/septic/solar). Notes Teton Co.'s low effective rate (~0.35-0.5%), the
Idaho ag-valuation retention lever (63-604, gated on CC&Rs allowing ag use),
and WUI insurance as the escalating risk.


Claude-Session: https://claude.ai/code/session_01Xxu7aLEZbdzmUJPZjmgRxA

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/driggs/construction-estimate.xlsx
+++ b/driggs/construction-estimate.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Cost Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Operating Cost" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,6 +108,18 @@
       <color rgb="005F6B70"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005F6B70"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -167,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -229,6 +242,26 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -325,6 +358,26 @@
     <comment ref="D34" authorId="0" shapeId="0">
       <text>
         <t>$500 simple/efficient to $750 sleek w/ big glass. Single-story adds cost per sf.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>estimate</author>
+  </authors>
+  <commentList>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Median effective rate in Teton County is 0.35%. A full-market second home with no homeowner exemption pays the levy rate; 0.5% is a reasonable planning midpoint.</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>Idaho §63-604: platting alone doesn't end ag status. Keep the balance in qualifying ag use (&gt;5 ac, $1,000+ ag revenue) and it stays ag-valued — UNLESS CC&amp;Rs prohibit ag use.</t>
       </text>
     </comment>
   </commentList>
@@ -1211,8 +1264,466 @@
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Annual Operating Cost — What It Costs to RUN the Place</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>First-estimate carrying cost at the end of each phase. 2026 dollars. Edit blue cells. See notes at right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>TAX &amp; RESERVE ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Effective property-tax rate</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Teton Co. median effective 0.35%; use 0.5% for a full-market second home. Verify w/ Treasurer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Assessed improvements — end of Phase 1</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>ADU + garage market value (~build cost proxy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Assessed improvements — end of Phase 2</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>+ main house; total improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Assessed homesite land (taxed portion)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>~1 ac at market IF the balance stays ag-valued (§63-604). Whole parcel ~$500k if not farmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Major repair/replacement reserve</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>% of improvement value set aside yearly for roof/siding/systems (sinking fund, not cash spent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ANNUAL COST</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>(end of phase)</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>ADU + garage</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>full build-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Property tax</t>
+        </is>
+      </c>
+      <c r="C13" s="17">
+        <f>(C6+C8)*C5</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>(C7+C8)*C5</f>
+        <v/>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Low rate, but scales with what's built</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Insurance (WUI / high-value)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Wildfire-exposed; market hardening — a real risk line</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Electricity (Fall River, net of solar)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>900</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>$39/mo access fee; solar offsets much of the geo load</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Propane (cooking / backup / fireplace)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Optional; minimal if fully electric</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Internet (Starlink / rural)</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>~$120/mo; same both phases</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Trash / recycling</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Rural hauler or county transfer station</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Snow removal (driveway)</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Long rural drive, heavy Teton snow, all winter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Shared road maintenance</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Crossed Arrows road easement (per CC&amp;Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Landscape / defensible space</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>WUI defensible-space upkeep; low-maint. design helps</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Well / septic / HVAC servicing</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>700</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Septic pump ~3–5 yr; well &amp; geo annual service</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Cash operating subtotal</t>
+        </is>
+      </c>
+      <c r="C23" s="19">
+        <f>SUM(C13:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>SUM(D13:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Major repair/replacement reserve</t>
+        </is>
+      </c>
+      <c r="C24" s="17">
+        <f>C6*C9</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>C7*C9</f>
+        <v/>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Sinking fund for long-cycle replacements</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Caretaking / property mgmt (if 2nd home)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Optional; winter check-ins for an absentee home</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>TOTAL ALL-IN / YEAR</t>
+        </is>
+      </c>
+      <c r="C26" s="28">
+        <f>C23+C24+C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="28">
+        <f>D23+D24+D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="27" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>≈ per month</t>
+        </is>
+      </c>
+      <c r="C27" s="35">
+        <f>C26/12</f>
+        <v/>
+      </c>
+      <c r="D27" s="35">
+        <f>D26/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>Cash-only (excl. reserve &amp; caretaking)</t>
+        </is>
+      </c>
+      <c r="C29" s="37">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="D29" s="37">
+        <f>D23</f>
+        <v/>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>What actually leaves your pocket each year</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56" customHeight="1">
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>First-estimate only. The big three — property tax, insurance, and the maintenance reserve — all scale with the VALUE of what's built, so Phase 2 roughly triples the carrying cost even though the utility bills stay modest (well + septic + solar = no water/sewer bill and a small net electric bill). Verify the tax rate &amp; assessed value with the Teton County Assessor/Treasurer, get a real insurance quote (WUI underwriting is tightening), and confirm ag-valuation retention against the CC&amp;Rs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
driggs: set ~$750k land anchor (Nevin's read); mark price boundaries
Nevin volunteered Lot 3 is worth ~$750k based on recent nearby closings —
a developer-informed current-value read (~$31k/ac, the entitled/amenity
premium). Adopt ~$750k as the working land anchor: bump the cost model land
line $0.5M -> $0.75M (total incl land ~$4.85M; xlsx land input updated).
Record Mike's boundaries: do NOT ask Nevin about price and do not negotiate
through him (deal is with Caldwell/Lot 3); drop the 'what Caldwell paid in
2023' chase. Updates open-items (item 1 + valuation anchors), dossier §15,
and the construction estimate (.md + .xlsx).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xxu7aLEZbdzmUJPZjmgRxA
</commit_message>
<xml_diff>
--- a/driggs/construction-estimate.xlsx
+++ b/driggs/construction-estimate.xlsx
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
@@ -1264,8 +1264,8 @@
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B1:F1"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
driggs: set ~$750k land anchor (Nevin's read); mark price boundaries (#99)
Nevin volunteered Lot 3 is worth ~$750k based on recent nearby closings —
a developer-informed current-value read (~$31k/ac, the entitled/amenity
premium). Adopt ~$750k as the working land anchor: bump the cost model land
line $0.5M -> $0.75M (total incl land ~$4.85M; xlsx land input updated).
Record Mike's boundaries: do NOT ask Nevin about price and do not negotiate
through him (deal is with Caldwell/Lot 3); drop the 'what Caldwell paid in
2023' chase. Updates open-items (item 1 + valuation anchors), dossier §15,
and the construction estimate (.md + .xlsx).


Claude-Session: https://claude.ai/code/session_01Xxu7aLEZbdzmUJPZjmgRxA

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/driggs/construction-estimate.xlsx
+++ b/driggs/construction-estimate.xlsx
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
@@ -1264,8 +1264,8 @@
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B1:F1"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>